<commit_message>
[feat] Phase 5 step 2: gross earnings / months worked HFP columns
Optional Wages and Contributions columns feeding etEarnings_in / etMonths_in
(plan §4.2). Absent gross earnings falls back to anticipated wages with a
deferral-year warning; absent months worked defaults to 12 when countable
earnings are positive. Spec fca2f2cf was reviewed and its must-fixes applied
before this commit. UI help, Documentation, PARAMETERS, example workbooks.
</commit_message>
<xml_diff>
--- a/examples/HFP_alex+jamie.xlsx
+++ b/examples/HFP_alex+jamie.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,60 +432,70 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>gross earnings</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>months worked</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>other inc</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>net inv</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>taxable ctrb</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>401k ctrb</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Roth 401k ctrb</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>IRA ctrb</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Roth IRA ctrb</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Roth conv</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Roth conv fixed</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>QCD</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>HSA ctrb</t>
         </is>
@@ -495,19 +505,33 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="n">
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="n">
         <v>6500</v>
       </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -515,19 +539,33 @@
       <c r="A3" t="n">
         <v>2022</v>
       </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="n">
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="n">
         <v>6500</v>
       </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -535,19 +573,33 @@
       <c r="A4" t="n">
         <v>2023</v>
       </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="n">
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="n">
         <v>7000</v>
       </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -564,13 +616,26 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="n">
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="n">
         <v>7000</v>
       </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -587,16 +652,28 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="n">
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="n">
         <v>7000</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
         <v>20000</v>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -613,13 +690,26 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
       <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
         <v>15000</v>
       </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -636,13 +726,26 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
       <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
         <v>15000</v>
       </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -659,13 +762,26 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="J9" t="n">
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
         <v>50000</v>
       </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -673,19 +789,33 @@
       <c r="A10" t="n">
         <v>2029</v>
       </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="n">
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
         <v>50000</v>
       </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -693,16 +823,31 @@
       <c r="A11" t="n">
         <v>2030</v>
       </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -710,16 +855,31 @@
       <c r="A12" t="n">
         <v>2031</v>
       </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -727,16 +887,31 @@
       <c r="A13" t="n">
         <v>2032</v>
       </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -744,16 +919,31 @@
       <c r="A14" t="n">
         <v>2033</v>
       </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -761,16 +951,31 @@
       <c r="A15" t="n">
         <v>2034</v>
       </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -778,16 +983,31 @@
       <c r="A16" t="n">
         <v>2035</v>
       </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -795,16 +1015,31 @@
       <c r="A17" t="n">
         <v>2036</v>
       </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -812,16 +1047,31 @@
       <c r="A18" t="n">
         <v>2037</v>
       </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -829,16 +1079,31 @@
       <c r="A19" t="n">
         <v>2038</v>
       </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -846,16 +1111,31 @@
       <c r="A20" t="n">
         <v>2039</v>
       </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -863,16 +1143,31 @@
       <c r="A21" t="n">
         <v>2040</v>
       </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -880,16 +1175,31 @@
       <c r="A22" t="n">
         <v>2041</v>
       </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="L22" t="n">
-        <v>0</v>
-      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -897,16 +1207,31 @@
       <c r="A23" t="n">
         <v>2042</v>
       </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -914,16 +1239,31 @@
       <c r="A24" t="n">
         <v>2043</v>
       </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -931,16 +1271,31 @@
       <c r="A25" t="n">
         <v>2044</v>
       </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -948,16 +1303,31 @@
       <c r="A26" t="n">
         <v>2045</v>
       </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
       <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -965,16 +1335,31 @@
       <c r="A27" t="n">
         <v>2046</v>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -982,16 +1367,31 @@
       <c r="A28" t="n">
         <v>2047</v>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -999,16 +1399,31 @@
       <c r="A29" t="n">
         <v>2048</v>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
       <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1016,16 +1431,31 @@
       <c r="A30" t="n">
         <v>2049</v>
       </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1033,16 +1463,31 @@
       <c r="A31" t="n">
         <v>2050</v>
       </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
       <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1050,16 +1495,31 @@
       <c r="A32" t="n">
         <v>2051</v>
       </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
       <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1067,16 +1527,31 @@
       <c r="A33" t="n">
         <v>2052</v>
       </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="L33" t="n">
-        <v>0</v>
-      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
       <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1084,16 +1559,31 @@
       <c r="A34" t="n">
         <v>2053</v>
       </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="L34" t="n">
-        <v>0</v>
-      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
       <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1101,16 +1591,31 @@
       <c r="A35" t="n">
         <v>2054</v>
       </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="L35" t="n">
-        <v>0</v>
-      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
       <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1118,16 +1623,31 @@
       <c r="A36" t="n">
         <v>2055</v>
       </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="L36" t="n">
-        <v>0</v>
-      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1142,7 +1662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:P39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1158,60 +1678,70 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>gross earnings</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>months worked</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>other inc</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>net inv</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>taxable ctrb</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>401k ctrb</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Roth 401k ctrb</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>IRA ctrb</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Roth IRA ctrb</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Roth conv</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Roth conv fixed</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>QCD</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>HSA ctrb</t>
         </is>
@@ -1221,19 +1751,33 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="n">
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="n">
         <v>4000</v>
       </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1241,19 +1785,33 @@
       <c r="A3" t="n">
         <v>2022</v>
       </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" t="n">
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
         <v>4000</v>
       </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1261,19 +1819,33 @@
       <c r="A4" t="n">
         <v>2023</v>
       </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="n">
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="n">
         <v>4000</v>
       </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1290,13 +1862,26 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="J5" t="n">
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
         <v>12000</v>
       </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1313,13 +1898,26 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="I6" t="n">
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="n">
         <v>5000</v>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1336,10 +1934,24 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -1356,10 +1968,24 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -1376,10 +2002,24 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1387,16 +2027,31 @@
       <c r="A10" t="n">
         <v>2029</v>
       </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1404,16 +2059,31 @@
       <c r="A11" t="n">
         <v>2030</v>
       </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1421,16 +2091,31 @@
       <c r="A12" t="n">
         <v>2031</v>
       </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1438,16 +2123,31 @@
       <c r="A13" t="n">
         <v>2032</v>
       </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1455,16 +2155,31 @@
       <c r="A14" t="n">
         <v>2033</v>
       </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1472,16 +2187,31 @@
       <c r="A15" t="n">
         <v>2034</v>
       </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1489,16 +2219,31 @@
       <c r="A16" t="n">
         <v>2035</v>
       </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1506,16 +2251,31 @@
       <c r="A17" t="n">
         <v>2036</v>
       </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1523,16 +2283,31 @@
       <c r="A18" t="n">
         <v>2037</v>
       </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1540,16 +2315,31 @@
       <c r="A19" t="n">
         <v>2038</v>
       </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1557,16 +2347,31 @@
       <c r="A20" t="n">
         <v>2039</v>
       </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1574,16 +2379,31 @@
       <c r="A21" t="n">
         <v>2040</v>
       </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1591,16 +2411,31 @@
       <c r="A22" t="n">
         <v>2041</v>
       </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="L22" t="n">
-        <v>0</v>
-      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1608,16 +2443,31 @@
       <c r="A23" t="n">
         <v>2042</v>
       </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1625,16 +2475,31 @@
       <c r="A24" t="n">
         <v>2043</v>
       </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1642,16 +2507,31 @@
       <c r="A25" t="n">
         <v>2044</v>
       </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1659,16 +2539,31 @@
       <c r="A26" t="n">
         <v>2045</v>
       </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
       <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1676,16 +2571,31 @@
       <c r="A27" t="n">
         <v>2046</v>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1693,16 +2603,31 @@
       <c r="A28" t="n">
         <v>2047</v>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1710,16 +2635,31 @@
       <c r="A29" t="n">
         <v>2048</v>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
       <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1727,16 +2667,31 @@
       <c r="A30" t="n">
         <v>2049</v>
       </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1744,16 +2699,31 @@
       <c r="A31" t="n">
         <v>2050</v>
       </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
       <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1761,16 +2731,31 @@
       <c r="A32" t="n">
         <v>2051</v>
       </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
       <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1778,16 +2763,31 @@
       <c r="A33" t="n">
         <v>2052</v>
       </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="L33" t="n">
-        <v>0</v>
-      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
       <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1795,16 +2795,31 @@
       <c r="A34" t="n">
         <v>2053</v>
       </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="L34" t="n">
-        <v>0</v>
-      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
       <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1812,16 +2827,31 @@
       <c r="A35" t="n">
         <v>2054</v>
       </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="L35" t="n">
-        <v>0</v>
-      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
       <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1829,16 +2859,31 @@
       <c r="A36" t="n">
         <v>2055</v>
       </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="L36" t="n">
-        <v>0</v>
-      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1846,16 +2891,31 @@
       <c r="A37" t="n">
         <v>2056</v>
       </c>
+      <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
         <v>0</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
       </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1863,16 +2923,31 @@
       <c r="A38" t="n">
         <v>2057</v>
       </c>
+      <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
         <v>0</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
-      <c r="L38" t="n">
-        <v>0</v>
-      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1880,16 +2955,31 @@
       <c r="A39" t="n">
         <v>2058</v>
       </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="n">
         <v>0</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
       </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
       <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1906,10 +2996,6 @@
   </sheetPr>
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>